<commit_message>
Inclusão do campo de Telefone e testes
</commit_message>
<xml_diff>
--- a/SME.ConectaFormacao.Infra.Dados/Templates/Template_Relatorio_Inscritos_Por_Formacao.xlsx
+++ b/SME.ConectaFormacao.Infra.Dados/Templates/Template_Relatorio_Inscritos_Por_Formacao.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="30720" windowHeight="8400" tabRatio="500"/>
+    <workbookView windowWidth="30720" windowHeight="7800" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
   <si>
     <t>CONECTA</t>
   </si>
@@ -152,6 +152,9 @@
     <t>Situação da inscrição</t>
   </si>
   <si>
+    <t>Telefone</t>
+  </si>
+  <si>
     <t>Situação da conclusão</t>
   </si>
   <si>
@@ -225,6 +228,9 @@
   </si>
   <si>
     <t>{{inscritos.SituacaoInscricao}}</t>
+  </si>
+  <si>
+    <t>{{inscritos.Telefone}}</t>
   </si>
   <si>
     <t>{{inscritos.SituacaoConclusao}}</t>
@@ -1568,7 +1574,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:BA8"/>
+  <dimension ref="A1:BB8"/>
   <sheetFormatPr defaultColWidth="11.537037037037" defaultRowHeight="15" customHeight="1" outlineLevelRow="7"/>
   <cols>
     <col min="1" max="15" width="17.287037037037" customWidth="1"/>
@@ -1583,7 +1589,7 @@
     <col min="36" max="50" width="8.67592592592593" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:53">
+    <row r="1" customHeight="1" spans="1:54">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1637,7 +1643,7 @@
       <c r="AW1" s="2"/>
       <c r="AX1" s="2"/>
     </row>
-    <row r="2" ht="23.25" customHeight="1" spans="1:53">
+    <row r="2" ht="23.25" customHeight="1" spans="1:54">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1689,7 +1695,7 @@
       <c r="AW2" s="2"/>
       <c r="AX2" s="2"/>
     </row>
-    <row r="3" ht="18" spans="1:53">
+    <row r="3" ht="18" spans="1:54">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -1743,7 +1749,7 @@
       <c r="AW3" s="3"/>
       <c r="AX3" s="3"/>
     </row>
-    <row r="4" ht="14.4" spans="1:53">
+    <row r="4" ht="14.4" spans="1:54">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -1795,7 +1801,7 @@
       <c r="AW4" s="1"/>
       <c r="AX4" s="1"/>
     </row>
-    <row r="5" ht="14.4" spans="1:53">
+    <row r="5" ht="14.4" spans="1:54">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -1813,7 +1819,7 @@
       </c>
       <c r="J5" s="5"/>
     </row>
-    <row r="6" ht="14.4" spans="1:53">
+    <row r="6" ht="14.4" spans="1:54">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -1850,7 +1856,7 @@
       <c r="AH6" s="1"/>
       <c r="AI6" s="1"/>
     </row>
-    <row r="7" ht="23.85" customHeight="1" spans="1:53">
+    <row r="7" ht="23.85" customHeight="1" spans="1:54">
       <c r="A7" s="6" t="s">
         <v>5</v>
       </c>
@@ -1921,144 +1927,150 @@
       <c r="AF7" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="AG7" s="11" t="s">
+      <c r="AG7" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="AH7" s="11"/>
+      <c r="AH7" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="AI7" s="11"/>
-      <c r="AJ7" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="AK7" s="11"/>
+      <c r="AJ7" s="11"/>
+      <c r="AK7" s="11" t="s">
+        <v>26</v>
+      </c>
       <c r="AL7" s="11"/>
-      <c r="AM7" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="AN7" s="13"/>
+      <c r="AM7" s="11"/>
+      <c r="AN7" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="AO7" s="13"/>
-      <c r="AP7" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="AQ7" s="13"/>
+      <c r="AP7" s="13"/>
+      <c r="AQ7" s="13" t="s">
+        <v>28</v>
+      </c>
       <c r="AR7" s="13"/>
       <c r="AS7" s="13"/>
-      <c r="AT7" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="AU7" s="13"/>
+      <c r="AT7" s="13"/>
+      <c r="AU7" s="13" t="s">
+        <v>29</v>
+      </c>
       <c r="AV7" s="13"/>
       <c r="AW7" s="13"/>
-      <c r="AX7" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="AY7" s="13"/>
+      <c r="AX7" s="13"/>
+      <c r="AY7" s="13" t="s">
+        <v>30</v>
+      </c>
       <c r="AZ7" s="13"/>
       <c r="BA7" s="13"/>
+      <c r="BB7" s="13"/>
     </row>
-    <row r="8" ht="33" customHeight="1" spans="1:53">
+    <row r="8" ht="33" customHeight="1" spans="1:54">
       <c r="A8" s="14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D8" s="15"/>
       <c r="E8" s="15"/>
       <c r="F8" s="16" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G8" s="16"/>
       <c r="H8" s="15" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I8" s="15"/>
       <c r="J8" s="15"/>
       <c r="K8" s="15" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="L8" s="15"/>
       <c r="M8" s="15"/>
       <c r="N8" s="17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="O8" s="17"/>
       <c r="P8" s="18" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Q8" s="15" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="R8" s="15" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="S8" s="15" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T8" s="15"/>
       <c r="U8" s="15" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="V8" s="15"/>
       <c r="W8" s="15" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="X8" s="15" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Y8" s="15"/>
       <c r="Z8" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AA8" s="15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AB8" s="16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="AC8" s="16"/>
       <c r="AD8" s="16"/>
       <c r="AE8" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="AF8" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="AG8" s="16" t="s">
+      <c r="AF8" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="AH8" s="16"/>
+      <c r="AG8" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="AH8" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="AI8" s="16"/>
-      <c r="AJ8" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="AK8" s="16"/>
+      <c r="AJ8" s="16"/>
+      <c r="AK8" s="16" t="s">
+        <v>52</v>
+      </c>
       <c r="AL8" s="16"/>
-      <c r="AM8" s="20" t="s">
-        <v>51</v>
-      </c>
-      <c r="AN8" s="20"/>
+      <c r="AM8" s="16"/>
+      <c r="AN8" s="20" t="s">
+        <v>53</v>
+      </c>
       <c r="AO8" s="20"/>
-      <c r="AP8" s="19" t="s">
-        <v>52</v>
-      </c>
-      <c r="AQ8" s="19"/>
+      <c r="AP8" s="20"/>
+      <c r="AQ8" s="19" t="s">
+        <v>54</v>
+      </c>
       <c r="AR8" s="19"/>
       <c r="AS8" s="19"/>
-      <c r="AT8" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="AU8" s="20"/>
+      <c r="AT8" s="19"/>
+      <c r="AU8" s="20" t="s">
+        <v>55</v>
+      </c>
       <c r="AV8" s="20"/>
       <c r="AW8" s="20"/>
-      <c r="AX8" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="AY8" s="16"/>
+      <c r="AX8" s="20"/>
+      <c r="AY8" s="16" t="s">
+        <v>56</v>
+      </c>
       <c r="AZ8" s="16"/>
       <c r="BA8" s="16"/>
+      <c r="BB8" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="38">
@@ -2077,12 +2089,12 @@
     <mergeCell ref="U7:V7"/>
     <mergeCell ref="X7:Y7"/>
     <mergeCell ref="AB7:AD7"/>
-    <mergeCell ref="AG7:AI7"/>
-    <mergeCell ref="AJ7:AL7"/>
-    <mergeCell ref="AM7:AO7"/>
-    <mergeCell ref="AP7:AS7"/>
-    <mergeCell ref="AT7:AW7"/>
-    <mergeCell ref="AX7:BA7"/>
+    <mergeCell ref="AH7:AJ7"/>
+    <mergeCell ref="AK7:AM7"/>
+    <mergeCell ref="AN7:AP7"/>
+    <mergeCell ref="AQ7:AT7"/>
+    <mergeCell ref="AU7:AX7"/>
+    <mergeCell ref="AY7:BB7"/>
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="F8:G8"/>
     <mergeCell ref="H8:J8"/>
@@ -2092,12 +2104,12 @@
     <mergeCell ref="U8:V8"/>
     <mergeCell ref="X8:Y8"/>
     <mergeCell ref="AB8:AD8"/>
-    <mergeCell ref="AG8:AI8"/>
-    <mergeCell ref="AJ8:AL8"/>
-    <mergeCell ref="AM8:AO8"/>
-    <mergeCell ref="AP8:AS8"/>
-    <mergeCell ref="AT8:AW8"/>
-    <mergeCell ref="AX8:BA8"/>
+    <mergeCell ref="AH8:AJ8"/>
+    <mergeCell ref="AK8:AM8"/>
+    <mergeCell ref="AN8:AP8"/>
+    <mergeCell ref="AQ8:AT8"/>
+    <mergeCell ref="AU8:AX8"/>
+    <mergeCell ref="AY8:BB8"/>
     <mergeCell ref="A1:C5"/>
     <mergeCell ref="D1:AX2"/>
   </mergeCells>

</xml_diff>

<commit_message>
Adicionar campo de data e hora de inscrição no relatório de inscritos por formação + testes
</commit_message>
<xml_diff>
--- a/SME.ConectaFormacao.Infra.Dados/Templates/Template_Relatorio_Inscritos_Por_Formacao.xlsx
+++ b/SME.ConectaFormacao.Infra.Dados/Templates/Template_Relatorio_Inscritos_Por_Formacao.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="30720" windowHeight="7800" tabRatio="500"/>
+    <workbookView windowWidth="30720" windowHeight="8400" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
     <t>CONECTA</t>
   </si>
@@ -152,6 +152,12 @@
     <t>Situação da inscrição</t>
   </si>
   <si>
+    <t>Data da inscrição</t>
+  </si>
+  <si>
+    <t>Hora da inscrição</t>
+  </si>
+  <si>
     <t>Telefone</t>
   </si>
   <si>
@@ -230,10 +236,10 @@
     <t>{{inscritos.SituacaoInscricao}}</t>
   </si>
   <si>
-    <t>{{inscritos.Telefone}}</t>
-  </si>
-  <si>
-    <t>{{inscritos.SituacaoConclusao}}</t>
+    <t>{{inscritos.DataInscricao}}</t>
+  </si>
+  <si>
+    <t>{{inscritos.HoraInscricao}}</t>
   </si>
   <si>
     <t>{{inscritos.Email}}</t>
@@ -1574,7 +1580,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:BB8"/>
+  <dimension ref="A1:BD8"/>
   <sheetFormatPr defaultColWidth="11.537037037037" defaultRowHeight="15" customHeight="1" outlineLevelRow="7"/>
   <cols>
     <col min="1" max="15" width="17.287037037037" customWidth="1"/>
@@ -1589,7 +1595,7 @@
     <col min="36" max="50" width="8.67592592592593" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:54">
+    <row r="1" customHeight="1" spans="1:56">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1643,7 +1649,7 @@
       <c r="AW1" s="2"/>
       <c r="AX1" s="2"/>
     </row>
-    <row r="2" ht="23.25" customHeight="1" spans="1:54">
+    <row r="2" ht="23.25" customHeight="1" spans="1:56">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1695,7 +1701,7 @@
       <c r="AW2" s="2"/>
       <c r="AX2" s="2"/>
     </row>
-    <row r="3" ht="18" spans="1:54">
+    <row r="3" ht="18" spans="1:56">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -1749,7 +1755,7 @@
       <c r="AW3" s="3"/>
       <c r="AX3" s="3"/>
     </row>
-    <row r="4" ht="14.4" spans="1:54">
+    <row r="4" ht="14.4" spans="1:56">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -1801,7 +1807,7 @@
       <c r="AW4" s="1"/>
       <c r="AX4" s="1"/>
     </row>
-    <row r="5" ht="14.4" spans="1:54">
+    <row r="5" ht="14.4" spans="1:56">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -1819,7 +1825,7 @@
       </c>
       <c r="J5" s="5"/>
     </row>
-    <row r="6" ht="14.4" spans="1:54">
+    <row r="6" ht="14.4" spans="1:56">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -1856,7 +1862,7 @@
       <c r="AH6" s="1"/>
       <c r="AI6" s="1"/>
     </row>
-    <row r="7" ht="23.85" customHeight="1" spans="1:54">
+    <row r="7" ht="23.85" customHeight="1" spans="1:56">
       <c r="A7" s="6" t="s">
         <v>5</v>
       </c>
@@ -1924,149 +1930,155 @@
       <c r="AE7" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="AF7" s="12" t="s">
+      <c r="AF7" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="AG7" s="12" t="s">
+      <c r="AG7" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="AH7" s="11" t="s">
+      <c r="AH7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="AI7" s="11"/>
-      <c r="AJ7" s="11"/>
-      <c r="AK7" s="11" t="s">
+      <c r="AI7" s="12" t="s">
         <v>26</v>
       </c>
+      <c r="AJ7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AK7" s="11"/>
       <c r="AL7" s="11"/>
-      <c r="AM7" s="11"/>
-      <c r="AN7" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="AO7" s="13"/>
-      <c r="AP7" s="13"/>
-      <c r="AQ7" s="13" t="s">
+      <c r="AM7" s="11" t="s">
         <v>28</v>
       </c>
+      <c r="AN7" s="11"/>
+      <c r="AO7" s="11"/>
+      <c r="AP7" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="AQ7" s="13"/>
       <c r="AR7" s="13"/>
-      <c r="AS7" s="13"/>
+      <c r="AS7" s="13" t="s">
+        <v>30</v>
+      </c>
       <c r="AT7" s="13"/>
-      <c r="AU7" s="13" t="s">
-        <v>29</v>
-      </c>
+      <c r="AU7" s="13"/>
       <c r="AV7" s="13"/>
-      <c r="AW7" s="13"/>
+      <c r="AW7" s="13" t="s">
+        <v>31</v>
+      </c>
       <c r="AX7" s="13"/>
-      <c r="AY7" s="13" t="s">
-        <v>30</v>
-      </c>
+      <c r="AY7" s="13"/>
       <c r="AZ7" s="13"/>
-      <c r="BA7" s="13"/>
+      <c r="BA7" s="13" t="s">
+        <v>32</v>
+      </c>
       <c r="BB7" s="13"/>
+      <c r="BC7" s="13"/>
+      <c r="BD7" s="13"/>
     </row>
-    <row r="8" ht="33" customHeight="1" spans="1:54">
+    <row r="8" ht="33" customHeight="1" spans="1:56">
       <c r="A8" s="14" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D8" s="15"/>
       <c r="E8" s="15"/>
       <c r="F8" s="16" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G8" s="16"/>
       <c r="H8" s="15" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="I8" s="15"/>
       <c r="J8" s="15"/>
       <c r="K8" s="15" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="L8" s="15"/>
       <c r="M8" s="15"/>
       <c r="N8" s="17" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="O8" s="17"/>
       <c r="P8" s="18" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="Q8" s="15" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="R8" s="15" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="S8" s="15" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="T8" s="15"/>
       <c r="U8" s="15" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="V8" s="15"/>
       <c r="W8" s="15" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="X8" s="15" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="Y8" s="15"/>
       <c r="Z8" s="19" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="AA8" s="15" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="AB8" s="16" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AC8" s="16"/>
       <c r="AD8" s="16"/>
       <c r="AE8" s="15" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="AF8" s="15" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AG8" s="19" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="AH8" s="16" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="AI8" s="16"/>
       <c r="AJ8" s="16"/>
       <c r="AK8" s="16" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="AL8" s="16"/>
       <c r="AM8" s="16"/>
       <c r="AN8" s="20" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="AO8" s="20"/>
       <c r="AP8" s="20"/>
       <c r="AQ8" s="19" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="AR8" s="19"/>
       <c r="AS8" s="19"/>
       <c r="AT8" s="19"/>
       <c r="AU8" s="20" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="AV8" s="20"/>
       <c r="AW8" s="20"/>
       <c r="AX8" s="20"/>
       <c r="AY8" s="16" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="AZ8" s="16"/>
       <c r="BA8" s="16"/>
@@ -2089,12 +2101,12 @@
     <mergeCell ref="U7:V7"/>
     <mergeCell ref="X7:Y7"/>
     <mergeCell ref="AB7:AD7"/>
-    <mergeCell ref="AH7:AJ7"/>
-    <mergeCell ref="AK7:AM7"/>
-    <mergeCell ref="AN7:AP7"/>
-    <mergeCell ref="AQ7:AT7"/>
-    <mergeCell ref="AU7:AX7"/>
-    <mergeCell ref="AY7:BB7"/>
+    <mergeCell ref="AJ7:AL7"/>
+    <mergeCell ref="AM7:AO7"/>
+    <mergeCell ref="AP7:AR7"/>
+    <mergeCell ref="AS7:AV7"/>
+    <mergeCell ref="AW7:AZ7"/>
+    <mergeCell ref="BA7:BD7"/>
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="F8:G8"/>
     <mergeCell ref="H8:J8"/>

</xml_diff>